<commit_message>
Mark the Town Centre Activation Value Model as in development
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/business-industry-trade/meanwhile-use-value-model-worked-example.xlsx
+++ b/business-industry-trade/meanwhile-use-value-model-worked-example.xlsx
@@ -794,7 +794,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Version 0.1, 23 October 2026 (pre-Budget; revise after the 28 October 2026 Budget)</t>
+          <t>In development. Version 0.1, 23 October 2026 (pre-Budget; revise after the 28 October 2026 Budget). Figures may change between versions</t>
         </is>
       </c>
     </row>
@@ -4453,7 +4453,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Version 0.1, 23 October 2026 (pre-Budget; revise after the 28 October 2026 Budget). Indicative appraisal following the MHCLG Appraisal Guide (2026), not a business case.</t>
+          <t>In development. Version 0.1, 23 October 2026 (pre-Budget; revise after the 28 October 2026 Budget). Figures may change between versions. Indicative appraisal following the MHCLG Appraisal Guide (2026), not a business case.</t>
         </is>
       </c>
     </row>

</xml_diff>